<commit_message>
Making changes to product listing , imp methods for better handling for diversified products verification
</commit_message>
<xml_diff>
--- a/eclipse-workspace/Intro/src/main/resources/data/Products.xlsx
+++ b/eclipse-workspace/Intro/src/main/resources/data/Products.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sagar\amazon-filter-e2e-automation\eclipse-workspace\Intro\src\main\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE56A58-DCAD-4D08-AFD2-CB4ABE4A6827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9163C9-CFB9-4EEA-81E4-3E9855272D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Products</t>
   </si>
@@ -36,7 +36,13 @@
     <t>Laptop</t>
   </si>
   <si>
-    <t>Pendriver</t>
+    <t>Tablet</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Smart Tv</t>
   </si>
 </sst>
 </file>
@@ -354,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -377,6 +383,16 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
RUnning all the tests with 3 prodcuts only
</commit_message>
<xml_diff>
--- a/eclipse-workspace/Intro/src/main/resources/data/Products.xlsx
+++ b/eclipse-workspace/Intro/src/main/resources/data/Products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sagar\amazon-filter-e2e-automation\eclipse-workspace\Intro\src\main\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9163C9-CFB9-4EEA-81E4-3E9855272D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61B921A-C918-4B65-8F90-F10234E96202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Products</t>
   </si>
@@ -37,12 +37,6 @@
   </si>
   <si>
     <t>Tablet</t>
-  </si>
-  <si>
-    <t>Monitor</t>
-  </si>
-  <si>
-    <t>Smart Tv</t>
   </si>
 </sst>
 </file>
@@ -360,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -383,16 +377,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>